<commit_message>
cloaim bonus key added
</commit_message>
<xml_diff>
--- a/setbet/locales-excel/en.xlsx
+++ b/setbet/locales-excel/en.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C521"/>
+  <dimension ref="A1:C522"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5125,12 +5125,12 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>tabs.active</t>
+          <t>tabs.claim</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Active Bonus</t>
+          <t>Claim Bonus</t>
         </is>
       </c>
     </row>
@@ -5142,12 +5142,12 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>tabs.unclaimed</t>
+          <t>tabs.active</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Unclaimed Bonus</t>
+          <t>Active Bonus</t>
         </is>
       </c>
     </row>
@@ -5159,12 +5159,12 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>tabs.redeemed</t>
+          <t>tabs.unclaimed</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Redeemed Bonus</t>
+          <t>Unclaimed Bonus</t>
         </is>
       </c>
     </row>
@@ -5176,12 +5176,12 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>noCampaigns</t>
+          <t>tabs.redeemed</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>No Campaigns available. Please check back later.</t>
+          <t>Redeemed Bonus</t>
         </is>
       </c>
     </row>
@@ -5193,12 +5193,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>campaignName</t>
+          <t>noCampaigns</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Campaign Name</t>
+          <t>No Campaigns available. Please check back later.</t>
         </is>
       </c>
     </row>
@@ -5210,12 +5210,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>campaignCode</t>
+          <t>campaignName</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Campaign Code</t>
+          <t>Campaign Name</t>
         </is>
       </c>
     </row>
@@ -5227,12 +5227,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>minOdds</t>
+          <t>campaignCode</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Min Odds</t>
+          <t>Campaign Code</t>
         </is>
       </c>
     </row>
@@ -5244,12 +5244,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>bonusAmount</t>
+          <t>minOdds</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Bonus Amount</t>
+          <t>Min Odds</t>
         </is>
       </c>
     </row>
@@ -5261,12 +5261,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>bonusPercentage</t>
+          <t>bonusAmount</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Bonus Percentage</t>
+          <t>Bonus Amount</t>
         </is>
       </c>
     </row>
@@ -5278,12 +5278,12 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>bonusPercentage</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Warning</t>
+          <t>Bonus Percentage</t>
         </is>
       </c>
     </row>
@@ -5295,12 +5295,12 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>cancelConfirm</t>
+          <t>warning</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Do you really want to cancel the bonus?</t>
+          <t>Warning</t>
         </is>
       </c>
     </row>
@@ -5312,12 +5312,12 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>promoCode</t>
+          <t>cancelConfirm</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Promo code</t>
+          <t>Do you really want to cancel the bonus?</t>
         </is>
       </c>
     </row>
@@ -5329,12 +5329,12 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>promoCodePlaceholder</t>
+          <t>promoCode</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Enter Promo code</t>
+          <t>Promo code</t>
         </is>
       </c>
     </row>
@@ -5346,12 +5346,12 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>claimIdle</t>
+          <t>promoCodePlaceholder</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Claim your Bonus</t>
+          <t>Enter Promo code</t>
         </is>
       </c>
     </row>
@@ -5363,12 +5363,12 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>claimLoading</t>
+          <t>claimIdle</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Claiming...</t>
+          <t>Claim your Bonus</t>
         </is>
       </c>
     </row>
@@ -5380,12 +5380,12 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>toasts.expireCampaignError</t>
+          <t>claimLoading</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Failed to expire campaign.</t>
+          <t>Claiming...</t>
         </is>
       </c>
     </row>
@@ -5397,12 +5397,12 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>toasts.campaignExpired</t>
+          <t>toasts.expireCampaignError</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Campaign Expired</t>
+          <t>Failed to expire campaign.</t>
         </is>
       </c>
     </row>
@@ -5414,29 +5414,29 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>toasts.claimError</t>
+          <t>toasts.campaignExpired</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Failed to claim Bonus.</t>
+          <t>Campaign Expired</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>kyc</t>
+          <t>bonus</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>toasts.claimError</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>KYC</t>
+          <t>Failed to claim Bonus.</t>
         </is>
       </c>
     </row>
@@ -5448,12 +5448,12 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>subtitle</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Update KYC</t>
+          <t>KYC</t>
         </is>
       </c>
     </row>
@@ -5465,12 +5465,12 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>documentTypeLabel</t>
+          <t>subtitle</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Document Type</t>
+          <t>Update KYC</t>
         </is>
       </c>
     </row>
@@ -5482,12 +5482,12 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>documentNumberLabel</t>
+          <t>documentTypeLabel</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Document Number</t>
+          <t>Document Type</t>
         </is>
       </c>
     </row>
@@ -5499,12 +5499,12 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>documentTypePlaceholder</t>
+          <t>documentNumberLabel</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Enter Document Type</t>
+          <t>Document Number</t>
         </is>
       </c>
     </row>
@@ -5516,12 +5516,12 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>documentNumberPlaceholder</t>
+          <t>documentTypePlaceholder</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Enter Document Number</t>
+          <t>Enter Document Type</t>
         </is>
       </c>
     </row>
@@ -5533,12 +5533,12 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>frontImageLabel</t>
+          <t>documentNumberPlaceholder</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Front Image</t>
+          <t>Enter Document Number</t>
         </is>
       </c>
     </row>
@@ -5550,12 +5550,12 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>backImageLabel</t>
+          <t>frontImageLabel</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Back Image</t>
+          <t>Front Image</t>
         </is>
       </c>
     </row>
@@ -5567,12 +5567,12 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>save</t>
+          <t>backImageLabel</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Save</t>
+          <t>Back Image</t>
         </is>
       </c>
     </row>
@@ -5584,12 +5584,12 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>saving</t>
+          <t>save</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Saving…</t>
+          <t>Save</t>
         </is>
       </c>
     </row>
@@ -5601,12 +5601,12 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>toastSuccess</t>
+          <t>saving</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Kyc Updated successfully.</t>
+          <t>Saving…</t>
         </is>
       </c>
     </row>
@@ -5618,12 +5618,12 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>toastError</t>
+          <t>toastSuccess</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Failed to update KYC.</t>
+          <t>Kyc Updated successfully.</t>
         </is>
       </c>
     </row>
@@ -5635,12 +5635,12 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>toastAlreadyVerified</t>
+          <t>toastError</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>KYC Already Verified</t>
+          <t>Failed to update KYC.</t>
         </is>
       </c>
     </row>
@@ -5652,12 +5652,12 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>toastPending</t>
+          <t>toastAlreadyVerified</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>KYC Status is Pending</t>
+          <t>KYC Already Verified</t>
         </is>
       </c>
     </row>
@@ -5669,12 +5669,12 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>toastRejected</t>
+          <t>toastPending</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>KYC Rejected</t>
+          <t>KYC Status is Pending</t>
         </is>
       </c>
     </row>
@@ -5686,12 +5686,12 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>validation.documentTypeRequired</t>
+          <t>toastRejected</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Please select a document type</t>
+          <t>KYC Rejected</t>
         </is>
       </c>
     </row>
@@ -5703,12 +5703,12 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>validation.documentNumberRequired</t>
+          <t>validation.documentTypeRequired</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Please enter your document number</t>
+          <t>Please select a document type</t>
         </is>
       </c>
     </row>
@@ -5720,12 +5720,12 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>validation.aadharInvalid</t>
+          <t>validation.documentNumberRequired</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Enter a valid 12-digit Aadhar Number</t>
+          <t>Please enter your document number</t>
         </is>
       </c>
     </row>
@@ -5737,12 +5737,12 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>validation.panInvalid</t>
+          <t>validation.aadharInvalid</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Enter a valid PAN Number</t>
+          <t>Enter a valid 12-digit Aadhar Number</t>
         </is>
       </c>
     </row>
@@ -5754,12 +5754,12 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>validation.frontImageRequired</t>
+          <t>validation.panInvalid</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Front image is required</t>
+          <t>Enter a valid PAN Number</t>
         </is>
       </c>
     </row>
@@ -5771,29 +5771,29 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>validation.backImageRequired</t>
+          <t>validation.frontImageRequired</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Back image is required</t>
+          <t>Front image is required</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>profile</t>
+          <t>kyc</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>validation.backImageRequired</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Back image is required</t>
         </is>
       </c>
     </row>
@@ -5805,12 +5805,12 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>yourPersonalData</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Your Personal Data</t>
+          <t>Profile</t>
         </is>
       </c>
     </row>
@@ -5822,12 +5822,12 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>updatePersonalData</t>
+          <t>yourPersonalData</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Update Personal Details</t>
+          <t>Your Personal Data</t>
         </is>
       </c>
     </row>
@@ -5839,12 +5839,12 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>fields.firstName</t>
+          <t>updatePersonalData</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>First Name</t>
+          <t>Update Personal Details</t>
         </is>
       </c>
     </row>
@@ -5856,12 +5856,12 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>fields.lastName</t>
+          <t>fields.firstName</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Last Name</t>
+          <t>First Name</t>
         </is>
       </c>
     </row>
@@ -5873,12 +5873,12 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>fields.userName</t>
+          <t>fields.lastName</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Username</t>
+          <t>Last Name</t>
         </is>
       </c>
     </row>
@@ -5890,12 +5890,12 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>fields.email</t>
+          <t>fields.userName</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Username</t>
         </is>
       </c>
     </row>
@@ -5907,12 +5907,12 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>fields.dateOfBirth</t>
+          <t>fields.email</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Date of Birth</t>
+          <t>Email</t>
         </is>
       </c>
     </row>
@@ -5924,12 +5924,12 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>fields.city</t>
+          <t>fields.dateOfBirth</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>Date of Birth</t>
         </is>
       </c>
     </row>
@@ -5941,12 +5941,12 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>fields.country</t>
+          <t>fields.city</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Country</t>
+          <t>City</t>
         </is>
       </c>
     </row>
@@ -5958,12 +5958,12 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>fields.state</t>
+          <t>fields.country</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Country</t>
         </is>
       </c>
     </row>
@@ -5975,12 +5975,12 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>fields.countryCode</t>
+          <t>fields.state</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Country Code</t>
+          <t>State</t>
         </is>
       </c>
     </row>
@@ -5992,12 +5992,12 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>fields.phone</t>
+          <t>fields.countryCode</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Phone Number</t>
+          <t>Country Code</t>
         </is>
       </c>
     </row>
@@ -6009,12 +6009,12 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>fields.address</t>
+          <t>fields.phone</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Address</t>
+          <t>Phone Number</t>
         </is>
       </c>
     </row>
@@ -6026,12 +6026,12 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>fields.currency</t>
+          <t>fields.address</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>Address</t>
         </is>
       </c>
     </row>
@@ -6043,12 +6043,12 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>fields.zipCode</t>
+          <t>fields.currency</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Zip Code</t>
+          <t>Currency</t>
         </is>
       </c>
     </row>
@@ -6060,12 +6060,12 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>validation.firstNameRequired</t>
+          <t>fields.zipCode</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Enter your first name</t>
+          <t>Zip Code</t>
         </is>
       </c>
     </row>
@@ -6077,12 +6077,12 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>validation.firstNameMaxLength</t>
+          <t>validation.firstNameRequired</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>First name cannot exceed 10 characters</t>
+          <t>Enter your first name</t>
         </is>
       </c>
     </row>
@@ -6094,12 +6094,12 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>validation.lastNameRequired</t>
+          <t>validation.firstNameMaxLength</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Enter your last name</t>
+          <t>First name cannot exceed 10 characters</t>
         </is>
       </c>
     </row>
@@ -6111,12 +6111,12 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>validation.lastNameMaxLength</t>
+          <t>validation.lastNameRequired</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Last name cannot exceed 10 characters</t>
+          <t>Enter your last name</t>
         </is>
       </c>
     </row>
@@ -6128,12 +6128,12 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>validation.emailPattern</t>
+          <t>validation.lastNameMaxLength</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Enter a valid email</t>
+          <t>Last name cannot exceed 10 characters</t>
         </is>
       </c>
     </row>
@@ -6145,12 +6145,12 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>validation.dobRequired</t>
+          <t>validation.emailPattern</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Select your DOB</t>
+          <t>Enter a valid email</t>
         </is>
       </c>
     </row>
@@ -6162,12 +6162,12 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>validation.countryCodeRequired</t>
+          <t>validation.dobRequired</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>Enter Country Code</t>
+          <t>Select your DOB</t>
         </is>
       </c>
     </row>
@@ -6179,12 +6179,12 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>validation.zipCodeRequired</t>
+          <t>validation.countryCodeRequired</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Please enter the pincode</t>
+          <t>Enter Country Code</t>
         </is>
       </c>
     </row>
@@ -6196,12 +6196,12 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>toasts.success</t>
+          <t>validation.zipCodeRequired</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Updated Player Details Successfully</t>
+          <t>Please enter the pincode</t>
         </is>
       </c>
     </row>
@@ -6213,29 +6213,29 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>toasts.error</t>
+          <t>toasts.success</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Failed to update player profile.</t>
+          <t>Updated Player Details Successfully</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>promotions</t>
+          <t>profile</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>noPromotions</t>
+          <t>toasts.error</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>No promotions available.</t>
+          <t>Failed to update player profile.</t>
         </is>
       </c>
     </row>
@@ -6247,29 +6247,29 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>imageAlt</t>
+          <t>noPromotions</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>promotion_card_image</t>
+          <t>No promotions available.</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>bankInfo</t>
+          <t>promotions</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>imageAlt</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Bank Information</t>
+          <t>promotion_card_image</t>
         </is>
       </c>
     </row>
@@ -6281,12 +6281,12 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>bankDetailsTitle</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Your Bank Data</t>
+          <t>Bank Information</t>
         </is>
       </c>
     </row>
@@ -6298,12 +6298,12 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>labels.accountNo</t>
+          <t>bankDetailsTitle</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Account No</t>
+          <t>Your Bank Data</t>
         </is>
       </c>
     </row>
@@ -6315,12 +6315,12 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>labels.bankName</t>
+          <t>labels.accountNo</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Bank Name</t>
+          <t>Account No</t>
         </is>
       </c>
     </row>
@@ -6332,12 +6332,12 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>labels.branchName</t>
+          <t>labels.bankName</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Branch Name</t>
+          <t>Bank Name</t>
         </is>
       </c>
     </row>
@@ -6349,12 +6349,12 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>labels.ifscCode</t>
+          <t>labels.branchName</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>IFSC Code</t>
+          <t>Branch Name</t>
         </is>
       </c>
     </row>
@@ -6366,12 +6366,12 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>labels.accountType</t>
+          <t>labels.ifscCode</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Account Type</t>
+          <t>IFSC Code</t>
         </is>
       </c>
     </row>
@@ -6383,12 +6383,12 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>labels.accountHolderName</t>
+          <t>labels.accountType</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Account Holder Name</t>
+          <t>Account Type</t>
         </is>
       </c>
     </row>
@@ -6400,12 +6400,12 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>labels.amount</t>
+          <t>labels.accountHolderName</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Account Holder Name</t>
         </is>
       </c>
     </row>
@@ -6417,12 +6417,12 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>labels.email</t>
+          <t>labels.amount</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Email Address</t>
+          <t>Amount</t>
         </is>
       </c>
     </row>
@@ -6434,12 +6434,12 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>placeholders.selectAccount</t>
+          <t>labels.email</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Select Bank Account</t>
+          <t>Email Address</t>
         </is>
       </c>
     </row>
@@ -6451,12 +6451,12 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>placeholders.enterAccountNo</t>
+          <t>placeholders.selectAccount</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>Enter Account Number</t>
+          <t>Select Bank Account</t>
         </is>
       </c>
     </row>
@@ -6468,12 +6468,12 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>placeholders.enterBankName</t>
+          <t>placeholders.enterAccountNo</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Enter Bank Name</t>
+          <t>Enter Account Number</t>
         </is>
       </c>
     </row>
@@ -6485,12 +6485,12 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>placeholders.enterAccountHolderName</t>
+          <t>placeholders.enterBankName</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Enter Account Holder Name</t>
+          <t>Enter Bank Name</t>
         </is>
       </c>
     </row>
@@ -6502,12 +6502,12 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>placeholders.enterBranchName</t>
+          <t>placeholders.enterAccountHolderName</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>Enter Branch Name</t>
+          <t>Enter Account Holder Name</t>
         </is>
       </c>
     </row>
@@ -6519,12 +6519,12 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>placeholders.enterIfscCode</t>
+          <t>placeholders.enterBranchName</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Enter IFSC Code</t>
+          <t>Enter Branch Name</t>
         </is>
       </c>
     </row>
@@ -6536,12 +6536,12 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>placeholders.enterAccountType</t>
+          <t>placeholders.enterIfscCode</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Enter Account Type</t>
+          <t>Enter IFSC Code</t>
         </is>
       </c>
     </row>
@@ -6553,12 +6553,12 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>placeholders.savings</t>
+          <t>placeholders.enterAccountType</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Savings</t>
+          <t>Enter Account Type</t>
         </is>
       </c>
     </row>
@@ -6570,12 +6570,12 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>placeholders.current</t>
+          <t>placeholders.savings</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Current</t>
+          <t>Savings</t>
         </is>
       </c>
     </row>
@@ -6587,12 +6587,12 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>validation.accountNoRequired</t>
+          <t>placeholders.current</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Account number is required</t>
+          <t>Current</t>
         </is>
       </c>
     </row>
@@ -6604,12 +6604,12 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>validation.accountNoNumbersOnly</t>
+          <t>validation.accountNoRequired</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Account Number must contain only numbers</t>
+          <t>Account number is required</t>
         </is>
       </c>
     </row>
@@ -6621,12 +6621,12 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>validation.accountNoMaxLength</t>
+          <t>validation.accountNoNumbersOnly</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Account Number cannot exceed 16 digits</t>
+          <t>Account Number must contain only numbers</t>
         </is>
       </c>
     </row>
@@ -6638,12 +6638,12 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>validation.accountNoDuplicate</t>
+          <t>validation.accountNoMaxLength</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>This account number is already registered.</t>
+          <t>Account Number cannot exceed 16 digits</t>
         </is>
       </c>
     </row>
@@ -6655,12 +6655,12 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>validation.bankNameRequired</t>
+          <t>validation.accountNoDuplicate</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Bank name is required</t>
+          <t>This account number is already registered.</t>
         </is>
       </c>
     </row>
@@ -6672,12 +6672,12 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>validation.accountHolderNameRequired</t>
+          <t>validation.bankNameRequired</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>Account holder name is required</t>
+          <t>Bank name is required</t>
         </is>
       </c>
     </row>
@@ -6689,12 +6689,12 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>validation.branchNameRequired</t>
+          <t>validation.accountHolderNameRequired</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Branch name is required</t>
+          <t>Account holder name is required</t>
         </is>
       </c>
     </row>
@@ -6706,12 +6706,12 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>validation.ifscCodeRequired</t>
+          <t>validation.branchNameRequired</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>IFSC Code is required</t>
+          <t>Branch name is required</t>
         </is>
       </c>
     </row>
@@ -6723,12 +6723,12 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>validation.ifscCodeInvalid</t>
+          <t>validation.ifscCodeRequired</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Enter a valid IFSC Code (4 letters + 7 digits)</t>
+          <t>IFSC Code is required</t>
         </is>
       </c>
     </row>
@@ -6740,12 +6740,12 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>validation.accountTypeRequired</t>
+          <t>validation.ifscCodeInvalid</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Please select an account type</t>
+          <t>Enter a valid IFSC Code (4 letters + 7 digits)</t>
         </is>
       </c>
     </row>
@@ -6757,12 +6757,12 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>validation.limitReached</t>
+          <t>validation.accountTypeRequired</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>You have reached the maximum limit of 5 bank accounts.</t>
+          <t>Please select an account type</t>
         </is>
       </c>
     </row>
@@ -6774,12 +6774,12 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>toasts.createSuccess</t>
+          <t>validation.limitReached</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Bank account created successfully.</t>
+          <t>You have reached the maximum limit of 5 bank accounts.</t>
         </is>
       </c>
     </row>
@@ -6791,12 +6791,12 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>toasts.createError</t>
+          <t>toasts.createSuccess</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>Failed to create bank account.</t>
+          <t>Bank account created successfully.</t>
         </is>
       </c>
     </row>
@@ -6808,12 +6808,12 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>toasts.updateSuccess</t>
+          <t>toasts.createError</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>Bank account updated successfully.</t>
+          <t>Failed to create bank account.</t>
         </is>
       </c>
     </row>
@@ -6825,12 +6825,12 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>toasts.updateError</t>
+          <t>toasts.updateSuccess</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Failed to update bank account</t>
+          <t>Bank account updated successfully.</t>
         </is>
       </c>
     </row>
@@ -6842,29 +6842,29 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>toasts.alreadyExists</t>
+          <t>toasts.updateError</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Bank Account Already Exists</t>
+          <t>Failed to update bank account</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>transactionHistory</t>
+          <t>bankInfo</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>toasts.alreadyExists</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>Transaction History</t>
+          <t>Bank Account Already Exists</t>
         </is>
       </c>
     </row>
@@ -6876,12 +6876,12 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>tabs.gameHistory</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>Game History</t>
+          <t>Transaction History</t>
         </is>
       </c>
     </row>
@@ -6893,12 +6893,12 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>tabs.depositSummary</t>
+          <t>tabs.gameHistory</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>Deposit Summary</t>
+          <t>Game History</t>
         </is>
       </c>
     </row>
@@ -6910,12 +6910,12 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>tabs.withdrawSummary</t>
+          <t>tabs.depositSummary</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Withdraw Summary</t>
+          <t>Deposit Summary</t>
         </is>
       </c>
     </row>
@@ -6927,12 +6927,12 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>tabs.allTransactions</t>
+          <t>tabs.withdrawSummary</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>All Transactions</t>
+          <t>Withdraw Summary</t>
         </is>
       </c>
     </row>
@@ -6944,12 +6944,12 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>transactionTable.columns.serialNo</t>
+          <t>tabs.allTransactions</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>SI NO</t>
+          <t>All Transactions</t>
         </is>
       </c>
     </row>
@@ -6961,12 +6961,12 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>transactionTable.columns.description</t>
+          <t>transactionTable.columns.serialNo</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>SI NO</t>
         </is>
       </c>
     </row>
@@ -6978,12 +6978,12 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>transactionTable.columns.gameName</t>
+          <t>transactionTable.columns.description</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Game Name</t>
+          <t>Description</t>
         </is>
       </c>
     </row>
@@ -6995,12 +6995,12 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>transactionTable.columns.startBalance</t>
+          <t>transactionTable.columns.gameName</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Start Balance</t>
+          <t>Game Name</t>
         </is>
       </c>
     </row>
@@ -7012,12 +7012,12 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>transactionTable.columns.amount</t>
+          <t>transactionTable.columns.startBalance</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Start Balance</t>
         </is>
       </c>
     </row>
@@ -7029,12 +7029,12 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>transactionTable.columns.endBalance</t>
+          <t>transactionTable.columns.amount</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>End Balance</t>
+          <t>Amount</t>
         </is>
       </c>
     </row>
@@ -7046,12 +7046,12 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>transactionTable.columns.timeStamp</t>
+          <t>transactionTable.columns.endBalance</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Time Stamp</t>
+          <t>End Balance</t>
         </is>
       </c>
     </row>
@@ -7063,12 +7063,12 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>transactionTable.columns.transactionStatus</t>
+          <t>transactionTable.columns.timeStamp</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Transaction Status</t>
+          <t>Time Stamp</t>
         </is>
       </c>
     </row>
@@ -7080,12 +7080,12 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>transactionTable.columns.providerName</t>
+          <t>transactionTable.columns.transactionStatus</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Provider Name</t>
+          <t>Transaction Status</t>
         </is>
       </c>
     </row>
@@ -7097,12 +7097,12 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>transactionTable.columns.transactionId</t>
+          <t>transactionTable.columns.providerName</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Transaction ID</t>
+          <t>Provider Name</t>
         </is>
       </c>
     </row>
@@ -7114,12 +7114,12 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>transactionTable.columns.gameTransactionId</t>
+          <t>transactionTable.columns.transactionId</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Game Transaction ID</t>
+          <t>Transaction ID</t>
         </is>
       </c>
     </row>
@@ -7131,12 +7131,12 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>transactionTable.columns.referenceId</t>
+          <t>transactionTable.columns.gameTransactionId</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Reference ID</t>
+          <t>Game Transaction ID</t>
         </is>
       </c>
     </row>
@@ -7148,12 +7148,12 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>transactionTable.columns.transactionNo</t>
+          <t>transactionTable.columns.referenceId</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>Transaction No</t>
+          <t>Reference ID</t>
         </is>
       </c>
     </row>
@@ -7165,12 +7165,12 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>transactionTable.columns.status</t>
+          <t>transactionTable.columns.transactionNo</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Transaction No</t>
         </is>
       </c>
     </row>
@@ -7182,12 +7182,12 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>transactionTable.pagination.rowsPerPage</t>
+          <t>transactionTable.columns.status</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Rows per page:</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -7199,12 +7199,12 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>transactionTable.pagination.prev</t>
+          <t>transactionTable.pagination.rowsPerPage</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Prev</t>
+          <t>Rows per page:</t>
         </is>
       </c>
     </row>
@@ -7216,12 +7216,12 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>transactionTable.pagination.next</t>
+          <t>transactionTable.pagination.prev</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Prev</t>
         </is>
       </c>
     </row>
@@ -7233,12 +7233,12 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.today</t>
+          <t>transactionTable.pagination.next</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>Next</t>
         </is>
       </c>
     </row>
@@ -7250,12 +7250,12 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.yesterday</t>
+          <t>transactionTable.dateSelector.today</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Yesterday</t>
+          <t>Today</t>
         </is>
       </c>
     </row>
@@ -7267,12 +7267,12 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.thisWeek</t>
+          <t>transactionTable.dateSelector.yesterday</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>This Week</t>
+          <t>Yesterday</t>
         </is>
       </c>
     </row>
@@ -7284,12 +7284,12 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.lastWeek</t>
+          <t>transactionTable.dateSelector.thisWeek</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Last Week</t>
+          <t>This Week</t>
         </is>
       </c>
     </row>
@@ -7301,12 +7301,12 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.thisMonth</t>
+          <t>transactionTable.dateSelector.lastWeek</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>This Month</t>
+          <t>Last Week</t>
         </is>
       </c>
     </row>
@@ -7318,12 +7318,12 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>transactionTable.dateSelector.lastMonth</t>
+          <t>transactionTable.dateSelector.thisMonth</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Last Month</t>
+          <t>This Month</t>
         </is>
       </c>
     </row>
@@ -7335,46 +7335,46 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>filters.allGames</t>
+          <t>transactionTable.dateSelector.lastMonth</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>All Games</t>
+          <t>Last Month</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>partners</t>
+          <t>transactionHistory</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>provider</t>
+          <t>filters.allGames</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Provider</t>
+          <t>All Games</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>header</t>
+          <t>partners</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>loginButton</t>
+          <t>provider</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>LOGIN</t>
+          <t>Provider</t>
         </is>
       </c>
     </row>
@@ -7386,12 +7386,12 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>registerButton</t>
+          <t>loginButton</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>REGISTER</t>
+          <t>LOGIN</t>
         </is>
       </c>
     </row>
@@ -7403,12 +7403,12 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>helloUser</t>
+          <t>registerButton</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Hello, {{userName}}</t>
+          <t>REGISTER</t>
         </is>
       </c>
     </row>
@@ -7420,12 +7420,12 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>balance</t>
+          <t>helloUser</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Balance</t>
+          <t>Hello, {{userName}}</t>
         </is>
       </c>
     </row>
@@ -7437,12 +7437,12 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>logout</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Logout</t>
+          <t>Balance</t>
         </is>
       </c>
     </row>
@@ -7454,29 +7454,29 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>toasts.logoutSuccess</t>
+          <t>logout</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>Logout successful</t>
+          <t>Logout</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>footer</t>
+          <t>header</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>socialLinks</t>
+          <t>toasts.logoutSuccess</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>Social Links</t>
+          <t>Logout successful</t>
         </is>
       </c>
     </row>
@@ -7488,12 +7488,12 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>contactAlt</t>
+          <t>socialLinks</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Social Links</t>
         </is>
       </c>
     </row>
@@ -7505,12 +7505,12 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>copyright</t>
+          <t>contactAlt</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>© Copyright 2026 {{brandName}}. All Rights Reserved.</t>
+          <t>Contact</t>
         </is>
       </c>
     </row>
@@ -7522,29 +7522,29 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>copyright</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>© Copyright 2026 {{brandName}}. All Rights Reserved.</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>theme</t>
+          <t>footer</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>switchToLight</t>
+          <t>version</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>Switch to Light Mode</t>
+          <t>Version</t>
         </is>
       </c>
     </row>
@@ -7556,46 +7556,46 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>switchToDark</t>
+          <t>switchToLight</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Switch to Dark Mode</t>
+          <t>Switch to Light Mode</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>notAuthorized</t>
+          <t>theme</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>switchToDark</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>You are not authorized to access this page.</t>
+          <t>Switch to Dark Mode</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>notAuthorized</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>code</t>
+          <t>message</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>You are not authorized to access this page.</t>
         </is>
       </c>
     </row>
@@ -7607,12 +7607,12 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>code</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Oops! Page Not Found</t>
+          <t>404</t>
         </is>
       </c>
     </row>
@@ -7624,29 +7624,29 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>The page you're looking for doesn't exist or has been moved. Let's get you back to where you belong.</t>
+          <t>Oops! Page Not Found</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>aboutSection</t>
+          <t>notFound</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>defaultTitle</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>ABOUT {{brandName}}</t>
+          <t>The page you're looking for doesn't exist or has been moved. Let's get you back to where you belong.</t>
         </is>
       </c>
     </row>
@@ -7658,29 +7658,29 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>bgAlt</t>
+          <t>defaultTitle</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>about background</t>
+          <t>ABOUT {{brandName}}</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>exploreFeatures</t>
+          <t>aboutSection</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>bgAlt</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>EXPLORE ALL FEATURES</t>
+          <t>about background</t>
         </is>
       </c>
     </row>
@@ -7692,12 +7692,12 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>downloadApplication</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>Download application</t>
+          <t>EXPLORE ALL FEATURES</t>
         </is>
       </c>
     </row>
@@ -7709,29 +7709,29 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>installApplication</t>
+          <t>downloadApplication</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>Install application</t>
+          <t>Download application</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>leaderboard</t>
+          <t>exploreFeatures</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>installApplication</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>Tournament</t>
+          <t>Install application</t>
         </is>
       </c>
     </row>
@@ -7743,12 +7743,12 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>termsAndConditions</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>Terms &amp; Conditions</t>
+          <t>Tournament</t>
         </is>
       </c>
     </row>
@@ -7760,12 +7760,12 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>myRank</t>
+          <t>termsAndConditions</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>My Rank</t>
+          <t>Terms &amp; Conditions</t>
         </is>
       </c>
     </row>
@@ -7777,12 +7777,12 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>start</t>
+          <t>myRank</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>Start</t>
+          <t>My Rank</t>
         </is>
       </c>
     </row>
@@ -7794,12 +7794,12 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>end</t>
+          <t>start</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>End</t>
+          <t>Start</t>
         </is>
       </c>
     </row>
@@ -7811,12 +7811,12 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>rank</t>
+          <t>end</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>Rank</t>
+          <t>End</t>
         </is>
       </c>
     </row>
@@ -7828,12 +7828,12 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>rank</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>Rank</t>
         </is>
       </c>
     </row>
@@ -7845,12 +7845,12 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>points</t>
+          <t>player</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Points</t>
+          <t>Player</t>
         </is>
       </c>
     </row>
@@ -7862,12 +7862,12 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>prize</t>
+          <t>points</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>Prize</t>
+          <t>Points</t>
         </is>
       </c>
     </row>
@@ -7879,12 +7879,12 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>noPlayersFound</t>
+          <t>prize</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>No players found</t>
+          <t>Prize</t>
         </is>
       </c>
     </row>
@@ -7896,12 +7896,12 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>noActiveTournaments</t>
+          <t>noPlayersFound</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>Currently no active tournaments</t>
+          <t>No players found</t>
         </is>
       </c>
     </row>
@@ -7913,29 +7913,29 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>trophyAlt</t>
+          <t>noActiveTournaments</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>trophy</t>
+          <t>Currently no active tournaments</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>ladder</t>
+          <t>leaderboard</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>loading</t>
+          <t>trophyAlt</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Loading your ladders…</t>
+          <t>trophy</t>
         </is>
       </c>
     </row>
@@ -7947,12 +7947,12 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>allMilestones</t>
+          <t>loading</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>All milestones</t>
+          <t>Loading your ladders…</t>
         </is>
       </c>
     </row>
@@ -7964,12 +7964,12 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>creditedInstantly</t>
+          <t>allMilestones</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>Credited instantly to your wallet</t>
+          <t>All milestones</t>
         </is>
       </c>
     </row>
@@ -7981,12 +7981,12 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>fullTermsApply</t>
+          <t>creditedInstantly</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>Full T&amp;C apply.</t>
+          <t>Credited instantly to your wallet</t>
         </is>
       </c>
     </row>
@@ -7998,12 +7998,12 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>simulatingProgress</t>
+          <t>fullTermsApply</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>Simulating progress</t>
+          <t>Full T&amp;C apply.</t>
         </is>
       </c>
     </row>
@@ -8015,12 +8015,12 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>simulateProgress</t>
+          <t>simulatingProgress</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>Simulate your progress</t>
+          <t>Simulating progress</t>
         </is>
       </c>
     </row>
@@ -8032,12 +8032,12 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>simulateBetAmount</t>
+          <t>simulateProgress</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>Simulate bet amount</t>
+          <t>Simulate your progress</t>
         </is>
       </c>
     </row>
@@ -8049,12 +8049,12 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>toNextReward</t>
+          <t>simulateBetAmount</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>to next reward</t>
+          <t>Simulate bet amount</t>
         </is>
       </c>
     </row>
@@ -8066,12 +8066,12 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>unlocked</t>
+          <t>toNextReward</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>unlocked</t>
+          <t>to next reward</t>
         </is>
       </c>
     </row>
@@ -8083,12 +8083,12 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>stillToEarn</t>
+          <t>unlocked</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>still to earn</t>
+          <t>unlocked</t>
         </is>
       </c>
     </row>
@@ -8100,12 +8100,12 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>nextReward</t>
+          <t>stillToEarn</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>Next reward</t>
+          <t>still to earn</t>
         </is>
       </c>
     </row>
@@ -8117,12 +8117,12 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>moreToUnlock</t>
+          <t>nextReward</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>more to unlock</t>
+          <t>Next reward</t>
         </is>
       </c>
     </row>
@@ -8134,12 +8134,12 @@
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>percentThere</t>
+          <t>moreToUnlock</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>of the way there</t>
+          <t>more to unlock</t>
         </is>
       </c>
     </row>
@@ -8151,12 +8151,12 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>allMilestonesCompletePre</t>
+          <t>percentThere</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>All milestones complete</t>
+          <t>of the way there</t>
         </is>
       </c>
     </row>
@@ -8168,12 +8168,12 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>allMilestonesCompletePost</t>
+          <t>allMilestonesCompletePre</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>earned!</t>
+          <t>All milestones complete</t>
         </is>
       </c>
     </row>
@@ -8185,12 +8185,12 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>bonusCredited</t>
+          <t>allMilestonesCompletePost</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>{{count}} bonus credited</t>
+          <t>earned!</t>
         </is>
       </c>
     </row>
@@ -8202,12 +8202,12 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>bonusesCredited</t>
+          <t>bonusCredited</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>{{count}} bonuses credited</t>
+          <t>{{count}} bonus credited</t>
         </is>
       </c>
     </row>
@@ -8219,12 +8219,12 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>milestoneName</t>
+          <t>bonusesCredited</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>{{name}} milestone</t>
+          <t>{{count}} bonuses credited</t>
         </is>
       </c>
     </row>
@@ -8236,12 +8236,12 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>creditedInstantlyLabel</t>
+          <t>milestoneName</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>Credited instantly</t>
+          <t>{{name}} milestone</t>
         </is>
       </c>
     </row>
@@ -8253,12 +8253,12 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>bonusEarnedLabel</t>
+          <t>creditedInstantlyLabel</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>Bonus earned</t>
+          <t>Credited instantly</t>
         </is>
       </c>
     </row>
@@ -8270,12 +8270,12 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>totalPossible</t>
+          <t>bonusEarnedLabel</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>total possible</t>
+          <t>Bonus earned</t>
         </is>
       </c>
     </row>
@@ -8287,12 +8287,12 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>creditedRewards</t>
+          <t>totalPossible</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>Credited rewards</t>
+          <t>total possible</t>
         </is>
       </c>
     </row>
@@ -8304,12 +8304,12 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>credited</t>
+          <t>creditedRewards</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>CREDITED</t>
+          <t>Credited rewards</t>
         </is>
       </c>
     </row>
@@ -8321,12 +8321,12 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>realMoney</t>
+          <t>credited</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>real money</t>
+          <t>CREDITED</t>
         </is>
       </c>
     </row>
@@ -8338,12 +8338,12 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>completedAt</t>
+          <t>realMoney</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>Completed at</t>
+          <t>real money</t>
         </is>
       </c>
     </row>
@@ -8355,12 +8355,12 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>tierPercentThere</t>
+          <t>completedAt</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>{{pct}}% there</t>
+          <t>Completed at</t>
         </is>
       </c>
     </row>
@@ -8372,12 +8372,12 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>cumulativeBets</t>
+          <t>tierPercentThere</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>cumulative bets</t>
+          <t>{{pct}}% there</t>
         </is>
       </c>
     </row>
@@ -8389,12 +8389,12 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>promotion</t>
+          <t>cumulativeBets</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>Bonus Ladder Promotion</t>
+          <t>cumulative bets</t>
         </is>
       </c>
     </row>
@@ -8406,12 +8406,12 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>termsAndConditions</t>
+          <t>promotion</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>Terms &amp; Conditions</t>
+          <t>Bonus Ladder Promotion</t>
         </is>
       </c>
     </row>
@@ -8423,12 +8423,12 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>termsDialogLabel</t>
+          <t>termsAndConditions</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>Bonus Ladder Terms &amp; Conditions</t>
+          <t>Terms &amp; Conditions</t>
         </is>
       </c>
     </row>
@@ -8440,12 +8440,12 @@
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>understandAndClose</t>
+          <t>termsDialogLabel</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>I understand — close</t>
+          <t>Bonus Ladder Terms &amp; Conditions</t>
         </is>
       </c>
     </row>
@@ -8457,12 +8457,12 @@
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>variants.deposit.placed</t>
+          <t>understandAndClose</t>
         </is>
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>deposited</t>
+          <t>I understand — close</t>
         </is>
       </c>
     </row>
@@ -8474,12 +8474,12 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>variants.deposit.totalPlacedShort</t>
+          <t>variants.deposit.placed</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>Total deposited</t>
+          <t>deposited</t>
         </is>
       </c>
     </row>
@@ -8491,12 +8491,12 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>variants.deposit.totalPlacedLong</t>
+          <t>variants.deposit.totalPlacedShort</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>Total deposited this campaign</t>
+          <t>Total deposited</t>
         </is>
       </c>
     </row>
@@ -8508,12 +8508,12 @@
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>variants.deposit.milestonesUnlocked</t>
+          <t>variants.deposit.totalPlacedLong</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>{{done}} of {{total}} milestones reached</t>
+          <t>Total deposited this campaign</t>
         </is>
       </c>
     </row>
@@ -8525,12 +8525,12 @@
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>variants.deposit.betMoreToUnlock</t>
+          <t>variants.deposit.milestonesUnlocked</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>Deposit</t>
+          <t>{{done}} of {{total}} milestones reached</t>
         </is>
       </c>
     </row>
@@ -8542,12 +8542,12 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>variants.deposit.noRewardsYet</t>
+          <t>variants.deposit.betMoreToUnlock</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>No rewards yet — make your first qualifying deposit</t>
+          <t>Deposit</t>
         </is>
       </c>
     </row>
@@ -8559,12 +8559,12 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>variants.deposit.cumulativeUnit</t>
+          <t>variants.deposit.noRewardsYet</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>cumulative deposits</t>
+          <t>No rewards yet — make your first qualifying deposit</t>
         </is>
       </c>
     </row>
@@ -8576,12 +8576,12 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>variants.deposit.keepGoing</t>
+          <t>variants.deposit.cumulativeUnit</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>Keep depositing →</t>
+          <t>cumulative deposits</t>
         </is>
       </c>
     </row>
@@ -8593,12 +8593,12 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>variants.deposit.overlayNextCta</t>
+          <t>variants.deposit.keepGoing</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>Deposit</t>
+          <t>Keep depositing →</t>
         </is>
       </c>
     </row>
@@ -8610,12 +8610,12 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>variants.bet.placed</t>
+          <t>variants.deposit.overlayNextCta</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>placed</t>
+          <t>Deposit</t>
         </is>
       </c>
     </row>
@@ -8627,12 +8627,12 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>variants.bet.totalPlacedShort</t>
+          <t>variants.bet.placed</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Total bets placed</t>
+          <t>placed</t>
         </is>
       </c>
     </row>
@@ -8644,12 +8644,12 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>variants.bet.totalPlacedLong</t>
+          <t>variants.bet.totalPlacedShort</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Total bets placed this campaign</t>
+          <t>Total bets placed</t>
         </is>
       </c>
     </row>
@@ -8661,12 +8661,12 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>variants.bet.milestonesUnlocked</t>
+          <t>variants.bet.totalPlacedLong</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>{{done}} of {{total}} milestones unlocked</t>
+          <t>Total bets placed this campaign</t>
         </is>
       </c>
     </row>
@@ -8678,12 +8678,12 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>variants.bet.betMoreToUnlock</t>
+          <t>variants.bet.milestonesUnlocked</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Bet</t>
+          <t>{{done}} of {{total}} milestones unlocked</t>
         </is>
       </c>
     </row>
@@ -8695,12 +8695,12 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>variants.bet.noRewardsYet</t>
+          <t>variants.bet.betMoreToUnlock</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>No rewards yet — place your first qualifying bet</t>
+          <t>Bet</t>
         </is>
       </c>
     </row>
@@ -8712,12 +8712,12 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>variants.bet.cumulativeUnit</t>
+          <t>variants.bet.noRewardsYet</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>cumulative bets</t>
+          <t>No rewards yet — place your first qualifying bet</t>
         </is>
       </c>
     </row>
@@ -8729,12 +8729,12 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>variants.bet.keepGoing</t>
+          <t>variants.bet.cumulativeUnit</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Keep betting →</t>
+          <t>cumulative bets</t>
         </is>
       </c>
     </row>
@@ -8746,12 +8746,12 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>variants.bet.overlayNextCta</t>
+          <t>variants.bet.keepGoing</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Bet</t>
+          <t>Keep betting →</t>
         </is>
       </c>
     </row>
@@ -8763,12 +8763,12 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>overlay.allMilestonesComplete</t>
+          <t>variants.bet.overlayNextCta</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>All milestones complete!</t>
+          <t>Bet</t>
         </is>
       </c>
     </row>
@@ -8780,12 +8780,12 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>overlay.milestoneUnlocked</t>
+          <t>overlay.allMilestonesComplete</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Milestone unlocked</t>
+          <t>All milestones complete!</t>
         </is>
       </c>
     </row>
@@ -8797,12 +8797,12 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>overlay.tierReached</t>
+          <t>overlay.milestoneUnlocked</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>{{name}} reached!</t>
+          <t>Milestone unlocked</t>
         </is>
       </c>
     </row>
@@ -8814,12 +8814,12 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>overlay.rolloverNote</t>
+          <t>overlay.tierReached</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Real money · Rollover: 1× · Never expires</t>
+          <t>{{name}} reached!</t>
         </is>
       </c>
     </row>
@@ -8831,12 +8831,12 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>overlay.nextMilestone</t>
+          <t>overlay.rolloverNote</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Next milestone — {{name}}</t>
+          <t>Real money · Rollover: 1× · Never expires</t>
         </is>
       </c>
     </row>
@@ -8848,12 +8848,12 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>overlay.betMore</t>
+          <t>overlay.nextMilestone</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Bet</t>
+          <t>Next milestone — {{name}}</t>
         </is>
       </c>
     </row>
@@ -8865,12 +8865,12 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>overlay.betMoreToEarn</t>
+          <t>overlay.betMore</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>more to earn</t>
+          <t>Bet</t>
         </is>
       </c>
     </row>
@@ -8882,12 +8882,12 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>overlay.allDoneTitle</t>
+          <t>overlay.betMoreToEarn</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>You've completed all milestones!</t>
+          <t>more to earn</t>
         </is>
       </c>
     </row>
@@ -8899,12 +8899,12 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>overlay.allDoneSubtitle</t>
+          <t>overlay.allDoneTitle</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>All bonuses have been credited to your wallet.</t>
+          <t>You've completed all milestones!</t>
         </is>
       </c>
     </row>
@@ -8916,12 +8916,12 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>overlay.viewLadder</t>
+          <t>overlay.allDoneSubtitle</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>View my ladder</t>
+          <t>All bonuses have been credited to your wallet.</t>
         </is>
       </c>
     </row>
@@ -8933,12 +8933,12 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>overlay.viewLadderArrow</t>
+          <t>overlay.viewLadder</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>View my ladder →</t>
+          <t>View my ladder</t>
         </is>
       </c>
     </row>
@@ -8950,12 +8950,12 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>achievement.milestoneUnlocked</t>
+          <t>overlay.viewLadderArrow</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>Milestone unlocked</t>
+          <t>View my ladder →</t>
         </is>
       </c>
     </row>
@@ -8967,29 +8967,29 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>achievement.tierAchieved</t>
+          <t>achievement.milestoneUnlocked</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>Tier achieved!</t>
+          <t>Milestone unlocked</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>jackpot</t>
+          <t>ladder</t>
         </is>
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>monthlyJackpot</t>
+          <t>achievement.tierAchieved</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>Monthly Jackpot</t>
+          <t>Tier achieved!</t>
         </is>
       </c>
     </row>
@@ -9001,12 +9001,12 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>monthlyJackpot</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>Jackpot Winners</t>
+          <t>Monthly Jackpot</t>
         </is>
       </c>
     </row>
@@ -9018,12 +9018,12 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>winner</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>Jackpot winner</t>
+          <t>Jackpot Winners</t>
         </is>
       </c>
     </row>
@@ -9035,12 +9035,12 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>congratulationDefault</t>
+          <t>winner</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>Congratulations — you're one of this month's jackpot winners!</t>
+          <t>Jackpot winner</t>
         </is>
       </c>
     </row>
@@ -9052,12 +9052,12 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>youWonThisMonthPre</t>
+          <t>congratulationDefault</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>You won</t>
+          <t>Congratulations — you're one of this month's jackpot winners!</t>
         </is>
       </c>
     </row>
@@ -9069,12 +9069,12 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>youWonThisMonthPost</t>
+          <t>youWonThisMonthPre</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>this month</t>
+          <t>You won</t>
         </is>
       </c>
     </row>
@@ -9086,12 +9086,12 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>loadError</t>
+          <t>youWonThisMonthPost</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>Couldn't load winners for {{month}}.</t>
+          <t>this month</t>
         </is>
       </c>
     </row>
@@ -9103,12 +9103,12 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>noWinners</t>
+          <t>loadError</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>No jackpot winners yet for {{month}}</t>
+          <t>Couldn't load winners for {{month}}.</t>
         </is>
       </c>
     </row>
@@ -9120,12 +9120,12 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>checkBack</t>
+          <t>noWinners</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>Check back after the next draw.</t>
+          <t>No jackpot winners yet for {{month}}</t>
         </is>
       </c>
     </row>
@@ -9137,12 +9137,12 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>loadMore</t>
+          <t>checkBack</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>Load more winners</t>
+          <t>Check back after the next draw.</t>
         </is>
       </c>
     </row>
@@ -9154,12 +9154,12 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>winnerCount</t>
+          <t>loadMore</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>{{count}} winner for {{month}}</t>
+          <t>Load more winners</t>
         </is>
       </c>
     </row>
@@ -9171,12 +9171,12 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>winnersCount</t>
+          <t>winnerCount</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>{{count}} winners for {{month}}</t>
+          <t>{{count}} winner for {{month}}</t>
         </is>
       </c>
     </row>
@@ -9188,12 +9188,12 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>previousMonth</t>
+          <t>winnersCount</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>Previous month</t>
+          <t>{{count}} winners for {{month}}</t>
         </is>
       </c>
     </row>
@@ -9205,12 +9205,12 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>nextMonth</t>
+          <t>previousMonth</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>Next month</t>
+          <t>Previous month</t>
         </is>
       </c>
     </row>
@@ -9222,12 +9222,12 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>backToThisMonth</t>
+          <t>nextMonth</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>Back to this month</t>
+          <t>Next month</t>
         </is>
       </c>
     </row>
@@ -9239,12 +9239,12 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>you</t>
+          <t>backToThisMonth</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>You</t>
+          <t>Back to this month</t>
         </is>
       </c>
     </row>
@@ -9256,12 +9256,12 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>youBadge</t>
+          <t>you</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>YOU</t>
+          <t>You</t>
         </is>
       </c>
     </row>
@@ -9273,10 +9273,27 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
+          <t>youBadge</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>YOU</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>jackpot</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
           <t>place</t>
         </is>
       </c>
-      <c r="C521" t="inlineStr">
+      <c r="C522" t="inlineStr">
         <is>
           <t>{{position}} place</t>
         </is>

</xml_diff>